<commit_message>
Rename Suasio to Logos everywhere
The temptation-rite Opera category is now Logos across player-facing
copy, the sim category id and modifier channel, constants, the panel
id, component and CSS classes, docs, design handoffs and the economy
spreadsheet. The category id is not persisted, so no save migration.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VWqHFY8XNSLKecEVdWMhug
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sins &amp; Devotion" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sigils" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Suasio" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Logos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Decimatio" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Indagatio &amp; Emptio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Maleficia" sheetId="7" state="visible" r:id="rId7"/>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F6" s="67" t="inlineStr">
         <is>
-          <t>+100% overall Suasio efficiency (mult) /lvl; unlocks Suasio actions and toggles</t>
+          <t>+100% overall Logos efficiency (mult) /lvl; unlocks Logos actions and toggles</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="D21" s="81" t="inlineStr">
         <is>
-          <t>-Suasio negative outcome chance</t>
+          <t>-Logos negative outcome chance</t>
         </is>
       </c>
       <c r="E21" s="61" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="D43" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> +chance to duplicate output of Suasio</t>
+          <t xml:space="preserve"> +chance to duplicate output of Logos</t>
         </is>
       </c>
       <c r="E43" s="61" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="D51" s="85" t="inlineStr">
         <is>
-          <t>+Stellar chance for Suasio</t>
+          <t>+Stellar chance for Logos</t>
         </is>
       </c>
       <c r="E51" s="61" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="D60" s="77" t="inlineStr">
         <is>
-          <t>+Suasio positive outcome chance</t>
+          <t>+Logos positive outcome chance</t>
         </is>
       </c>
       <c r="E60" s="61" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="D75" s="88" t="inlineStr">
         <is>
-          <t>+Suasio action efficiency</t>
+          <t>+Logos action efficiency</t>
         </is>
       </c>
       <c r="E75" s="61" t="inlineStr">
@@ -5069,7 +5069,7 @@
     <row r="1" ht="19.5" customHeight="1" s="57">
       <c r="A1" s="65" t="inlineStr">
         <is>
-          <t>Suasio — Tempting</t>
+          <t>Logos — Tempting</t>
         </is>
       </c>
     </row>
@@ -6733,7 +6733,7 @@
       </c>
       <c r="F13" s="67" t="inlineStr">
         <is>
-          <t>reveal Suasio distribution</t>
+          <t>reveal Logos distribution</t>
         </is>
       </c>
       <c r="G13" s="69" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="F23" s="67" t="inlineStr">
         <is>
-          <t>*1.66 Suasio efficiency</t>
+          <t>*1.66 Logos efficiency</t>
         </is>
       </c>
       <c r="G23" s="69" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="F28" s="67" t="inlineStr">
         <is>
-          <t>*1.33 Suasio efficiency</t>
+          <t>*1.33 Logos efficiency</t>
         </is>
       </c>
       <c r="G28" s="69" t="inlineStr">

</xml_diff>

<commit_message>
Rename Suasio to Logos everywhere (#160)
The temptation-rite Opera category is now Logos across player-facing
copy, the sim category id and modifier channel, constants, the panel
id, component and CSS classes, docs, design handoffs and the economy
spreadsheet. The category id is not persisted, so no save migration.


Claude-Session: https://claude.ai/code/session_01VWqHFY8XNSLKecEVdWMhug

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Panvitium_Economy_Template.xlsx
+++ b/docs/Panvitium_Economy_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Globals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sins &amp; Devotion" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sigils" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Suasio" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Logos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Decimatio" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Indagatio &amp; Emptio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Maleficia" sheetId="7" state="visible" r:id="rId7"/>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F6" s="67" t="inlineStr">
         <is>
-          <t>+100% overall Suasio efficiency (mult) /lvl; unlocks Suasio actions and toggles</t>
+          <t>+100% overall Logos efficiency (mult) /lvl; unlocks Logos actions and toggles</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="D21" s="81" t="inlineStr">
         <is>
-          <t>-Suasio negative outcome chance</t>
+          <t>-Logos negative outcome chance</t>
         </is>
       </c>
       <c r="E21" s="61" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="D43" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> +chance to duplicate output of Suasio</t>
+          <t xml:space="preserve"> +chance to duplicate output of Logos</t>
         </is>
       </c>
       <c r="E43" s="61" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="D51" s="85" t="inlineStr">
         <is>
-          <t>+Stellar chance for Suasio</t>
+          <t>+Stellar chance for Logos</t>
         </is>
       </c>
       <c r="E51" s="61" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="D60" s="77" t="inlineStr">
         <is>
-          <t>+Suasio positive outcome chance</t>
+          <t>+Logos positive outcome chance</t>
         </is>
       </c>
       <c r="E60" s="61" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="D75" s="88" t="inlineStr">
         <is>
-          <t>+Suasio action efficiency</t>
+          <t>+Logos action efficiency</t>
         </is>
       </c>
       <c r="E75" s="61" t="inlineStr">
@@ -5069,7 +5069,7 @@
     <row r="1" ht="19.5" customHeight="1" s="57">
       <c r="A1" s="65" t="inlineStr">
         <is>
-          <t>Suasio — Tempting</t>
+          <t>Logos — Tempting</t>
         </is>
       </c>
     </row>
@@ -6733,7 +6733,7 @@
       </c>
       <c r="F13" s="67" t="inlineStr">
         <is>
-          <t>reveal Suasio distribution</t>
+          <t>reveal Logos distribution</t>
         </is>
       </c>
       <c r="G13" s="69" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="F23" s="67" t="inlineStr">
         <is>
-          <t>*1.66 Suasio efficiency</t>
+          <t>*1.66 Logos efficiency</t>
         </is>
       </c>
       <c r="G23" s="69" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="F28" s="67" t="inlineStr">
         <is>
-          <t>*1.33 Suasio efficiency</t>
+          <t>*1.33 Logos efficiency</t>
         </is>
       </c>
       <c r="G28" s="69" t="inlineStr">

</xml_diff>